<commit_message>
Scan 2026-10-29 19:41 ET
</commit_message>
<xml_diff>
--- a/site/reversal_signals.xlsx
+++ b/site/reversal_signals.xlsx
@@ -2544,7 +2544,7 @@
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Topping tail forming at the high (tail 46% of range) | Time count 7: up bars since the last real down bar | RSI overbought (75)</t>
+          <t>Topping tail forming at the high (tail 47% of range) | Time count 7: up bars since the last real down bar | RSI overbought (75)</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -3107,20 +3107,20 @@
         <v>65.12</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>65.84999999999999</v>
+        <v>65.84</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>59.3</v>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
-          <t>Topping tail forming at the high (tail 61% of range) | Liquidity swept Major swing high @ 65.53</t>
+          <t>Topping tail forming at the high (tail 62% of range) | Liquidity swept Major swing high @ 65.53</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
-          <t>Topping tail forming at the high (tail 50% of range) | Time count 1: up bars since the last real down bar | Liquidity swept Prior week's high @ 326.27</t>
+          <t>Topping tail forming at the high (tail 51% of range) | Time count 1: up bars since the last real down bar | Liquidity swept Prior week's high @ 326.27</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -3875,10 +3875,10 @@
         <v>196.42</v>
       </c>
       <c r="J53" s="6" t="n">
-        <v>189.59</v>
+        <v>189.6</v>
       </c>
       <c r="K53" s="6" t="n">
-        <v>3.48</v>
+        <v>3.47</v>
       </c>
       <c r="L53" s="6" t="n">
         <v>3.18</v>
@@ -6633,7 +6633,7 @@
         <v>0.36</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="M96" s="2" t="n">
         <v>73.5</v>

</xml_diff>